<commit_message>
first commit from samantha pc
</commit_message>
<xml_diff>
--- a/Harlow/Harlow_MATERIAL_PRICES.xlsx
+++ b/Harlow/Harlow_MATERIAL_PRICES.xlsx
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="J2" s="7" t="n">
-        <v>46288.40787788149</v>
+        <v>46290.40927894228</v>
       </c>
     </row>
     <row r="3">
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="J3" s="7" t="n">
-        <v>46288.40787729045</v>
+        <v>46290.40927782433</v>
       </c>
     </row>
   </sheetData>

</xml_diff>